<commit_message>
Optimization - label checking, email content optimization
</commit_message>
<xml_diff>
--- a/version1/data/Candidates.xlsx
+++ b/version1/data/Candidates.xlsx
@@ -8,20 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keert\OneDrive\Desktop\KEERTHIRAJ\PROJECTS\Email-Automation\version1\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668D60B6-C682-4F03-813D-DD123D4E2FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CD41110-F69E-40B2-9156-3CE424223981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="376">
   <si>
     <t>Name</t>
   </si>
@@ -1117,6 +1119,42 @@
   </si>
   <si>
     <t>onim zsab qctw etxb</t>
+  </si>
+  <si>
+    <t>Abdullah Solaiman</t>
+  </si>
+  <si>
+    <t>absolaiman92@gmail.com</t>
+  </si>
+  <si>
+    <t>ncbj jifh wtij bjod</t>
+  </si>
+  <si>
+    <t>Keerthi Lanka</t>
+  </si>
+  <si>
+    <t>keerthilanka87@gmail.com</t>
+  </si>
+  <si>
+    <t>inop oyzm wkac rjmo</t>
+  </si>
+  <si>
+    <t>Manvitha</t>
+  </si>
+  <si>
+    <t>m.srimanvitha27@gmail.com</t>
+  </si>
+  <si>
+    <t>rvnn lpic jzwh wkqr</t>
+  </si>
+  <si>
+    <t>Mehul</t>
+  </si>
+  <si>
+    <t>mehulkkumar86@gmail.com</t>
+  </si>
+  <si>
+    <t>kqds geuf kwom cbnr</t>
   </si>
 </sst>
 </file>
@@ -1456,7 +1494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
@@ -1477,123 +1515,46 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>236</v>
+        <v>364</v>
       </c>
       <c r="B2" t="s">
-        <v>237</v>
+        <v>365</v>
       </c>
       <c r="C2" t="s">
-        <v>238</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>239</v>
+        <v>367</v>
       </c>
       <c r="B3" t="s">
-        <v>240</v>
+        <v>368</v>
       </c>
       <c r="C3" t="s">
-        <v>241</v>
+        <v>369</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>242</v>
+        <v>370</v>
       </c>
       <c r="B4" t="s">
-        <v>243</v>
+        <v>371</v>
       </c>
       <c r="C4" t="s">
-        <v>244</v>
+        <v>372</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>245</v>
+        <v>373</v>
       </c>
       <c r="B5" t="s">
-        <v>246</v>
+        <v>374</v>
       </c>
       <c r="C5" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>286</v>
-      </c>
-      <c r="B6" t="s">
-        <v>287</v>
-      </c>
-      <c r="C6" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>289</v>
-      </c>
-      <c r="B7" t="s">
-        <v>290</v>
-      </c>
-      <c r="C7" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>292</v>
-      </c>
-      <c r="B8" t="s">
-        <v>293</v>
-      </c>
-      <c r="C8" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>295</v>
-      </c>
-      <c r="B9" t="s">
-        <v>296</v>
-      </c>
-      <c r="C9" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>298</v>
-      </c>
-      <c r="B10" t="s">
-        <v>299</v>
-      </c>
-      <c r="C10" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>301</v>
-      </c>
-      <c r="B11" t="s">
-        <v>302</v>
-      </c>
-      <c r="C11" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>304</v>
-      </c>
-      <c r="B12" t="s">
-        <v>305</v>
-      </c>
-      <c r="C12" t="s">
-        <v>306</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -1602,6 +1563,146 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3444D549-B8D2-4ABB-BFAE-62045244F625}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C3" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B4" t="s">
+        <v>246</v>
+      </c>
+      <c r="C4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>286</v>
+      </c>
+      <c r="B5" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>289</v>
+      </c>
+      <c r="B6" t="s">
+        <v>290</v>
+      </c>
+      <c r="C6" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>292</v>
+      </c>
+      <c r="B7" t="s">
+        <v>293</v>
+      </c>
+      <c r="C7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>295</v>
+      </c>
+      <c r="B8" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>298</v>
+      </c>
+      <c r="B9" t="s">
+        <v>299</v>
+      </c>
+      <c r="C9" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>301</v>
+      </c>
+      <c r="B10" t="s">
+        <v>302</v>
+      </c>
+      <c r="C10" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B11" t="s">
+        <v>305</v>
+      </c>
+      <c r="C11" t="s">
+        <v>306</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF1C4F62-221A-4E4F-8CC0-1166BF273412}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C93615BE-0499-449D-BF80-AA6F427FA5DC}">
   <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>